<commit_message>
Update weekly competition report
</commit_message>
<xml_diff>
--- a/reports/schedule_report.xlsx
+++ b/reports/schedule_report.xlsx
@@ -7874,7 +7874,7 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>挑战杯丨第十五届“挑战杯”中国大学生创业计划竞赛培训交流云南站倒计时！</t>
+          <t>挑战杯丨第十五届“挑战杯”中国大学生创业计划竞赛培训交流河北站倒计时！</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiaozhanbei.net/article/15834/</t>
+          <t>https://www.tiaozhanbei.net/article/15837/</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -7948,7 +7948,7 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>挑战杯丨第十五届“挑战杯”中国大学生创业计划竞赛培训交流河北站倒计时！</t>
+          <t>挑战杯丨第十五届“挑战杯”中国大学生创业计划竞赛培训交流（云南站）顺利举办</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -7988,7 +7988,7 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiaozhanbei.net/article/15837/</t>
+          <t>https://www.tiaozhanbei.net/article/15838/</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -8022,7 +8022,7 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>挑战杯丨第十五届“挑战杯”中国大学生创业计划竞赛培训交流（云南站）顺利举办</t>
+          <t>挑战杯丨第十五届“挑战杯”中国大学生创业计划竞赛培训交流（河北站）顺利举办</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -8062,7 +8062,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiaozhanbei.net/article/15838/</t>
+          <t>https://www.tiaozhanbei.net/article/15839/</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -8096,7 +8096,7 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>挑战杯丨速来！“挑战杯”竞赛“学霸笔记”上新啦！（三）</t>
+          <t>挑战杯丨速来！“挑战杯”竞赛“学霸笔记”上新啦！（四）</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -8136,7 +8136,7 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://mp.weixin.qq.com/s/Iu5xv-Nhr9wm7kit8_404Q?scene=1&amp;click_id=5</t>
+          <t>https://mp.weixin.qq.com/s/my059Ww6twn2E5PeFiGWFg</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">

</xml_diff>